<commit_message>
Se realizó el Planning Poker
</commit_message>
<xml_diff>
--- a/ProductBacklog.xlsx
+++ b/ProductBacklog.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\usuario\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\usuario\Documents\Projects\FastOrder\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{065B4818-FE34-44F7-9D50-86371B739A21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5882FEF-7C27-4B81-A119-E2E0AA34DA16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{11D656E6-743B-4C56-A5A1-A6ADF0BA1430}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="255">
   <si>
     <t>Cómo</t>
   </si>
@@ -288,9 +288,6 @@
     <t>Dado que el mesero ha preparado un pedido</t>
   </si>
   <si>
-    <t>Cuando intenta confirmarlo sin haber indicado la mesa correspondiente</t>
-  </si>
-  <si>
     <t>Entonces el sistema debe mostrar un mensaje indicando que debe asociarse una mesa al pedido</t>
   </si>
   <si>
@@ -453,9 +450,6 @@
     <t>Dado que el administrador está realizando una búsqueda</t>
   </si>
   <si>
-    <t>Cuando consulgta un criterio que no corresponde a ningún pedido registrado</t>
-  </si>
-  <si>
     <t>Entonces el sistema debe informar que no existen resultados para ese filtro</t>
   </si>
   <si>
@@ -609,12 +603,6 @@
     <t>Consultar una lista de pedidos vacía</t>
   </si>
   <si>
-    <t>Dado que el cocinero consulta los pedidos</t>
-  </si>
-  <si>
-    <t>Cuando no existen pedidos registrados</t>
-  </si>
-  <si>
     <t>Entonces el sistema debe indicar que no hay pedidos pendientes</t>
   </si>
   <si>
@@ -700,6 +688,117 @@
   </si>
   <si>
     <t>Cuando agrega una nota que supera el número máximo de caracteres o contiene caracteres no permitidos</t>
+  </si>
+  <si>
+    <t>Consultar un pedido ya finalizado</t>
+  </si>
+  <si>
+    <t>Dado que el mesero accede al módulo de seguimiento de pedidos</t>
+  </si>
+  <si>
+    <t>Cuando consulta un pedido que ya fue entregado y cerrado</t>
+  </si>
+  <si>
+    <t>Cuando intenta consultar pero no existen pedidos registrados</t>
+  </si>
+  <si>
+    <t>Entonces el sistema debe mostrar que el pedido se encuentra finalizado</t>
+  </si>
+  <si>
+    <t>Consultar pedidos ya atendidos</t>
+  </si>
+  <si>
+    <t>Cuando consulta pedidos que ya fueron preparados o entregados</t>
+  </si>
+  <si>
+    <t>Entonces el sistema no debe mostrarlos como pedidos pendientes de cocina</t>
+  </si>
+  <si>
+    <t>Visualizar un pedido ya cancelado</t>
+  </si>
+  <si>
+    <t>Dado que el cajero accede al módulo de facturación</t>
+  </si>
+  <si>
+    <t>Cuando ve un pedido que fue cancelado previamente</t>
+  </si>
+  <si>
+    <t>Entonces el sistema debe informar que el pedido no está disponible para generar factura</t>
+  </si>
+  <si>
+    <t>Consultar un pedido cancelado</t>
+  </si>
+  <si>
+    <t>Dado que el mesero accede al módulo de seguimiento</t>
+  </si>
+  <si>
+    <t>Cuando consulta un pedido que fue cancelado</t>
+  </si>
+  <si>
+    <t>Entonces el sistema debe mostrar que el pedido se encuentra cancelado</t>
+  </si>
+  <si>
+    <t>Cuando irevisa e ntenta confirmarlo sin haber indicado la mesa correspondiente</t>
+  </si>
+  <si>
+    <t>Dado que el cocinero se encuentra en la pantalla de pedidos</t>
+  </si>
+  <si>
+    <t>Cuando consulta un criterio que no corresponde a ningún pedido registrado</t>
+  </si>
+  <si>
+    <t>Planning Poker</t>
+  </si>
+  <si>
+    <t>Complejidad</t>
+  </si>
+  <si>
+    <t>Justificación</t>
+  </si>
+  <si>
+    <t>Registrar un pedido implica varias validaciones y el aseguramiento de que la información quede guardada correctamente en la base de datos. Además, es una funcionalidad clave del flujo principal del sistema.</t>
+  </si>
+  <si>
+    <t>Seleccionar productos del menú tiene una complejidad media, ya que requiere validar disponibilidad y cantidades correctas. Aunque es una acción frecuente, su lógica no es tan alta como otras historias más integradas.</t>
+  </si>
+  <si>
+    <t>Revisar y confirmar el pedido exige validar que toda la información sea correcta antes de enviarlo. Tiene una dificultad media por los posibles errores que deben detectarse y corregirse.</t>
+  </si>
+  <si>
+    <t>Asociar una mesa al pedido requiere validar que la mesa exista y esté disponible. No es una tarea simple, pero tampoco involucra tanta complejidad como procesos de envío o facturación.</t>
+  </si>
+  <si>
+    <t>Enviar el pedido automáticamente a cocina implica comunicación entre módulos y que la información llegue en tiempo real.</t>
+  </si>
+  <si>
+    <t>Agregar notas especiales es una funcionalidad puntual y relativamente sencilla. Solo requiere capturar el texto, validarlo y mostrarlo correctamente a cocina.</t>
+  </si>
+  <si>
+    <t>Recibir el pedido con detalles claros en cocina consiste principalmente en visualizar información ya registrada. No requiere demasiada lógica adicional.</t>
+  </si>
+  <si>
+    <t>Revisar instrucciones especiales es una consulta directa dentro del detalle del pedido. Es una historia simple, enfocada más en mostrar información que en procesarla.</t>
+  </si>
+  <si>
+    <t>Consultar pedidos ordenados implica organizar la información de manera clara y útil para priorizar la preparación. Tiene complejidad media por la lógica de orden y visualización.</t>
+  </si>
+  <si>
+    <t>Mostrar al cajero los detalles completos del pedido es fundamental para facturar correctamente. Involucra precisión en productos, cantidades y valores, por lo que un error impactaría directamente en la venta.</t>
+  </si>
+  <si>
+    <t>Modificar una factura requiere controlar restricciones importantes, como impedir cambios en facturas pagadas o inválidas.</t>
+  </si>
+  <si>
+    <t>Consultar todos los pedidos registrados implica manejar listados, filtros y validaciones de búsqueda. Tiene una complejidad media al trabajar con bastante información histórica.</t>
+  </si>
+  <si>
+    <t>Modificar o cancelar un pedido afecta directamente el flujo operativo del sistema y requiere validar estados del pedido. Es una historia compleja por las reglas de negocio involucradas.</t>
+  </si>
+  <si>
+    <t>Generar reportes requiere consolidar información, aplicar filtros y presentar resultados útiles para el seguimiento de ventas. Su complejidad aumenta por el manejo de datos y la generación correcta del reporte.</t>
+  </si>
+  <si>
+    <t>Consultar el estado actual de un pedido requiere mostrar información actualizada y consistente según el avance del proceso.</t>
   </si>
 </sst>
 </file>
@@ -767,12 +866,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
+        <fgColor theme="5" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -869,11 +968,31 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -914,16 +1033,25 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -932,7 +1060,46 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -941,59 +1108,35 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1003,8 +1146,8 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFADCBFD"/>
       <color rgb="FFE3EEFF"/>
-      <color rgb="FFADCBFD"/>
     </mruColors>
   </colors>
   <extLst>
@@ -1323,7 +1466,7 @@
   <cols>
     <col min="1" max="1" width="19.6640625" style="5" customWidth="1"/>
     <col min="2" max="2" width="11.6640625" style="4" customWidth="1"/>
-    <col min="3" max="3" width="14.88671875" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.33203125" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="29.77734375" style="2" customWidth="1"/>
     <col min="5" max="5" width="29.109375" style="1" customWidth="1"/>
     <col min="6" max="6" width="13.33203125" style="9" customWidth="1"/>
@@ -1331,43 +1474,51 @@
     <col min="8" max="8" width="32.6640625" style="2" customWidth="1"/>
     <col min="9" max="9" width="31.5546875" style="2" customWidth="1"/>
     <col min="10" max="10" width="55.6640625" style="2" customWidth="1"/>
-    <col min="11" max="16384" width="11.5546875" style="1"/>
+    <col min="11" max="11" width="13.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="45.6640625" style="16" customWidth="1"/>
+    <col min="13" max="16384" width="11.5546875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="44" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="39"/>
-      <c r="E1" s="39"/>
-      <c r="F1" s="39"/>
-      <c r="G1" s="39"/>
-      <c r="H1" s="39"/>
-      <c r="I1" s="39"/>
-      <c r="J1" s="40"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
+      <c r="G1" s="45"/>
+      <c r="H1" s="45"/>
+      <c r="I1" s="45"/>
+      <c r="J1" s="45"/>
+      <c r="K1" s="45"/>
+      <c r="L1" s="48"/>
     </row>
     <row r="2" spans="1:23" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="35" t="s">
-        <v>165</v>
-      </c>
-      <c r="C2" s="35"/>
-      <c r="D2" s="35"/>
-      <c r="E2" s="35"/>
-      <c r="F2" s="35" t="s">
-        <v>166</v>
-      </c>
-      <c r="G2" s="35"/>
-      <c r="H2" s="35"/>
-      <c r="I2" s="35"/>
-      <c r="J2" s="35"/>
+      <c r="B2" s="33" t="s">
+        <v>163</v>
+      </c>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33" t="s">
+        <v>164</v>
+      </c>
+      <c r="G2" s="33"/>
+      <c r="H2" s="33"/>
+      <c r="I2" s="33"/>
+      <c r="J2" s="33"/>
+      <c r="K2" s="39" t="s">
+        <v>237</v>
+      </c>
+      <c r="L2" s="39"/>
     </row>
     <row r="3" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A3" s="25" t="s">
+      <c r="A3" s="24" t="s">
         <v>30</v>
       </c>
       <c r="B3" s="12" t="s">
@@ -1396,23 +1547,29 @@
       </c>
       <c r="J3" s="12" t="s">
         <v>8</v>
+      </c>
+      <c r="K3" s="40" t="s">
+        <v>238</v>
+      </c>
+      <c r="L3" s="17" t="s">
+        <v>239</v>
       </c>
       <c r="M3" s="6"/>
       <c r="N3" s="4"/>
       <c r="O3" s="4"/>
     </row>
     <row r="4" spans="1:23" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A4" s="25"/>
-      <c r="B4" s="36" t="s">
+      <c r="A4" s="24"/>
+      <c r="B4" s="34" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="27" t="s">
+      <c r="C4" s="26" t="s">
         <v>26</v>
       </c>
-      <c r="D4" s="26" t="s">
+      <c r="D4" s="25" t="s">
         <v>36</v>
       </c>
-      <c r="E4" s="26" t="s">
+      <c r="E4" s="25" t="s">
         <v>27</v>
       </c>
       <c r="F4" s="10">
@@ -1430,8 +1587,14 @@
       <c r="J4" s="3" t="s">
         <v>62</v>
       </c>
+      <c r="K4" s="41">
+        <v>8</v>
+      </c>
+      <c r="L4" s="27" t="s">
+        <v>240</v>
+      </c>
       <c r="M4" s="6"/>
-      <c r="N4" s="34"/>
+      <c r="N4" s="35"/>
       <c r="O4" s="4"/>
       <c r="S4" s="9"/>
       <c r="T4" s="2"/>
@@ -1440,11 +1603,11 @@
       <c r="W4" s="2"/>
     </row>
     <row r="5" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A5" s="25"/>
-      <c r="B5" s="36"/>
-      <c r="C5" s="27"/>
-      <c r="D5" s="26"/>
-      <c r="E5" s="26"/>
+      <c r="A5" s="24"/>
+      <c r="B5" s="34"/>
+      <c r="C5" s="26"/>
+      <c r="D5" s="25"/>
+      <c r="E5" s="25"/>
       <c r="F5" s="10">
         <v>2</v>
       </c>
@@ -1455,14 +1618,16 @@
         <v>60</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="J5" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="M5" s="24"/>
-      <c r="N5" s="34"/>
-      <c r="O5" s="34"/>
+      <c r="K5" s="42"/>
+      <c r="L5" s="28"/>
+      <c r="M5" s="23"/>
+      <c r="N5" s="35"/>
+      <c r="O5" s="35"/>
       <c r="S5" s="9"/>
       <c r="T5" s="2"/>
       <c r="U5" s="2"/>
@@ -1470,11 +1635,11 @@
       <c r="W5" s="2"/>
     </row>
     <row r="6" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A6" s="25"/>
-      <c r="B6" s="36"/>
-      <c r="C6" s="27"/>
-      <c r="D6" s="26"/>
-      <c r="E6" s="26"/>
+      <c r="A6" s="24"/>
+      <c r="B6" s="34"/>
+      <c r="C6" s="26"/>
+      <c r="D6" s="25"/>
+      <c r="E6" s="25"/>
       <c r="F6" s="10">
         <v>3</v>
       </c>
@@ -1485,14 +1650,16 @@
         <v>60</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="J6" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="M6" s="24"/>
-      <c r="N6" s="34"/>
-      <c r="O6" s="34"/>
+      <c r="K6" s="43"/>
+      <c r="L6" s="29"/>
+      <c r="M6" s="23"/>
+      <c r="N6" s="35"/>
+      <c r="O6" s="35"/>
       <c r="S6" s="9"/>
       <c r="T6" s="2"/>
       <c r="U6" s="2"/>
@@ -1500,32 +1667,34 @@
       <c r="W6" s="2"/>
     </row>
     <row r="7" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A7" s="25"/>
-      <c r="B7" s="18"/>
-      <c r="C7" s="19"/>
-      <c r="D7" s="19"/>
-      <c r="E7" s="19"/>
-      <c r="F7" s="19"/>
-      <c r="G7" s="19"/>
-      <c r="H7" s="19"/>
-      <c r="I7" s="19"/>
-      <c r="J7" s="20"/>
-      <c r="M7" s="24"/>
+      <c r="A7" s="24"/>
+      <c r="B7" s="21"/>
+      <c r="C7" s="22"/>
+      <c r="D7" s="22"/>
+      <c r="E7" s="22"/>
+      <c r="F7" s="22"/>
+      <c r="G7" s="22"/>
+      <c r="H7" s="22"/>
+      <c r="I7" s="22"/>
+      <c r="J7" s="22"/>
+      <c r="K7" s="22"/>
+      <c r="L7" s="46"/>
+      <c r="M7" s="23"/>
       <c r="N7" s="4"/>
-      <c r="O7" s="34"/>
+      <c r="O7" s="35"/>
     </row>
     <row r="8" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A8" s="25"/>
-      <c r="B8" s="36" t="s">
+      <c r="A8" s="24"/>
+      <c r="B8" s="34" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="27" t="s">
+      <c r="C8" s="26" t="s">
         <v>26</v>
       </c>
-      <c r="D8" s="26" t="s">
+      <c r="D8" s="25" t="s">
         <v>35</v>
       </c>
-      <c r="E8" s="26" t="s">
+      <c r="E8" s="25" t="s">
         <v>28</v>
       </c>
       <c r="F8" s="10">
@@ -1538,19 +1707,25 @@
         <v>67</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="J8" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="N8" s="34"/>
+      <c r="K8" s="41">
+        <v>5</v>
+      </c>
+      <c r="L8" s="27" t="s">
+        <v>241</v>
+      </c>
+      <c r="N8" s="35"/>
     </row>
     <row r="9" spans="1:23" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A9" s="25"/>
-      <c r="B9" s="36"/>
-      <c r="C9" s="27"/>
-      <c r="D9" s="26"/>
-      <c r="E9" s="26"/>
+      <c r="A9" s="24"/>
+      <c r="B9" s="34"/>
+      <c r="C9" s="26"/>
+      <c r="D9" s="25"/>
+      <c r="E9" s="25"/>
       <c r="F9" s="10">
         <v>2</v>
       </c>
@@ -1561,21 +1736,23 @@
         <v>67</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="J9" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="M9" s="24"/>
-      <c r="N9" s="34"/>
-      <c r="O9" s="34"/>
+      <c r="K9" s="42"/>
+      <c r="L9" s="28"/>
+      <c r="M9" s="23"/>
+      <c r="N9" s="35"/>
+      <c r="O9" s="35"/>
     </row>
     <row r="10" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A10" s="25"/>
-      <c r="B10" s="36"/>
-      <c r="C10" s="27"/>
-      <c r="D10" s="26"/>
-      <c r="E10" s="26"/>
+      <c r="A10" s="24"/>
+      <c r="B10" s="34"/>
+      <c r="C10" s="26"/>
+      <c r="D10" s="25"/>
+      <c r="E10" s="25"/>
       <c r="F10" s="10">
         <v>3</v>
       </c>
@@ -1586,42 +1763,46 @@
         <v>73</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="J10" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="M10" s="24"/>
-      <c r="N10" s="34"/>
-      <c r="O10" s="34"/>
+      <c r="K10" s="43"/>
+      <c r="L10" s="29"/>
+      <c r="M10" s="23"/>
+      <c r="N10" s="35"/>
+      <c r="O10" s="35"/>
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A11" s="25"/>
-      <c r="B11" s="18"/>
-      <c r="C11" s="19"/>
-      <c r="D11" s="19"/>
-      <c r="E11" s="19"/>
-      <c r="F11" s="19"/>
-      <c r="G11" s="19"/>
-      <c r="H11" s="19"/>
-      <c r="I11" s="19"/>
-      <c r="J11" s="20"/>
-      <c r="M11" s="24"/>
+      <c r="A11" s="24"/>
+      <c r="B11" s="21"/>
+      <c r="C11" s="22"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="22"/>
+      <c r="F11" s="22"/>
+      <c r="G11" s="22"/>
+      <c r="H11" s="22"/>
+      <c r="I11" s="22"/>
+      <c r="J11" s="22"/>
+      <c r="K11" s="22"/>
+      <c r="L11" s="46"/>
+      <c r="M11" s="23"/>
       <c r="N11" s="7"/>
-      <c r="O11" s="34"/>
+      <c r="O11" s="35"/>
     </row>
     <row r="12" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A12" s="25"/>
-      <c r="B12" s="36" t="s">
+      <c r="A12" s="24"/>
+      <c r="B12" s="34" t="s">
         <v>12</v>
       </c>
-      <c r="C12" s="27" t="s">
+      <c r="C12" s="26" t="s">
         <v>26</v>
       </c>
-      <c r="D12" s="26" t="s">
+      <c r="D12" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="E12" s="26" t="s">
+      <c r="E12" s="25" t="s">
         <v>32</v>
       </c>
       <c r="F12" s="10">
@@ -1639,14 +1820,20 @@
       <c r="J12" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="N12" s="34"/>
+      <c r="K12" s="41">
+        <v>5</v>
+      </c>
+      <c r="L12" s="27" t="s">
+        <v>242</v>
+      </c>
+      <c r="N12" s="35"/>
     </row>
     <row r="13" spans="1:23" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A13" s="25"/>
-      <c r="B13" s="36"/>
-      <c r="C13" s="27"/>
-      <c r="D13" s="26"/>
-      <c r="E13" s="26"/>
+      <c r="A13" s="24"/>
+      <c r="B13" s="34"/>
+      <c r="C13" s="26"/>
+      <c r="D13" s="25"/>
+      <c r="E13" s="25"/>
       <c r="F13" s="10">
         <v>2</v>
       </c>
@@ -1657,21 +1844,23 @@
         <v>80</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="J13" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="M13" s="24"/>
-      <c r="N13" s="34"/>
-      <c r="O13" s="34"/>
+      <c r="K13" s="42"/>
+      <c r="L13" s="28"/>
+      <c r="M13" s="23"/>
+      <c r="N13" s="35"/>
+      <c r="O13" s="35"/>
     </row>
     <row r="14" spans="1:23" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A14" s="25"/>
-      <c r="B14" s="36"/>
-      <c r="C14" s="27"/>
-      <c r="D14" s="26"/>
-      <c r="E14" s="26"/>
+      <c r="A14" s="24"/>
+      <c r="B14" s="34"/>
+      <c r="C14" s="26"/>
+      <c r="D14" s="25"/>
+      <c r="E14" s="25"/>
       <c r="F14" s="10">
         <v>3</v>
       </c>
@@ -1682,1126 +1871,1343 @@
         <v>83</v>
       </c>
       <c r="I14" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="J14" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="J14" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="M14" s="24"/>
-      <c r="N14" s="34"/>
-      <c r="O14" s="34"/>
+      <c r="K14" s="43"/>
+      <c r="L14" s="29"/>
+      <c r="M14" s="23"/>
+      <c r="N14" s="35"/>
+      <c r="O14" s="35"/>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A15" s="25"/>
-      <c r="B15" s="21"/>
-      <c r="C15" s="22"/>
-      <c r="D15" s="22"/>
-      <c r="E15" s="22"/>
-      <c r="F15" s="22"/>
-      <c r="G15" s="22"/>
-      <c r="H15" s="22"/>
-      <c r="I15" s="22"/>
-      <c r="J15" s="23"/>
-      <c r="M15" s="24"/>
+      <c r="A15" s="24"/>
+      <c r="B15" s="37"/>
+      <c r="C15" s="38"/>
+      <c r="D15" s="38"/>
+      <c r="E15" s="38"/>
+      <c r="F15" s="38"/>
+      <c r="G15" s="38"/>
+      <c r="H15" s="38"/>
+      <c r="I15" s="38"/>
+      <c r="J15" s="38"/>
+      <c r="K15" s="38"/>
+      <c r="L15" s="47"/>
+      <c r="M15" s="23"/>
       <c r="N15" s="9"/>
-      <c r="O15" s="34"/>
+      <c r="O15" s="35"/>
     </row>
     <row r="16" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A16" s="25"/>
-      <c r="B16" s="31" t="s">
+      <c r="A16" s="24"/>
+      <c r="B16" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="C16" s="27" t="s">
+      <c r="C16" s="26" t="s">
         <v>26</v>
       </c>
-      <c r="D16" s="28" t="s">
-        <v>205</v>
-      </c>
-      <c r="E16" s="28" t="s">
-        <v>206</v>
+      <c r="D16" s="27" t="s">
+        <v>201</v>
+      </c>
+      <c r="E16" s="27" t="s">
+        <v>202</v>
       </c>
       <c r="F16" s="10">
         <v>1</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I16" s="3" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>209</v>
-      </c>
-      <c r="M16" s="24"/>
+        <v>205</v>
+      </c>
+      <c r="K16" s="41">
+        <v>5</v>
+      </c>
+      <c r="L16" s="27" t="s">
+        <v>243</v>
+      </c>
+      <c r="M16" s="23"/>
       <c r="N16" s="9"/>
-      <c r="O16" s="34"/>
+      <c r="O16" s="35"/>
     </row>
     <row r="17" spans="1:15" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A17" s="25"/>
-      <c r="B17" s="32"/>
-      <c r="C17" s="27"/>
-      <c r="D17" s="29"/>
-      <c r="E17" s="29"/>
+      <c r="A17" s="24"/>
+      <c r="B17" s="31"/>
+      <c r="C17" s="26"/>
+      <c r="D17" s="28"/>
+      <c r="E17" s="28"/>
       <c r="F17" s="10">
         <v>2</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>213</v>
-      </c>
-      <c r="M17" s="24"/>
+        <v>209</v>
+      </c>
+      <c r="K17" s="42"/>
+      <c r="L17" s="28"/>
+      <c r="M17" s="23"/>
       <c r="N17" s="9"/>
-      <c r="O17" s="34"/>
+      <c r="O17" s="35"/>
     </row>
     <row r="18" spans="1:15" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A18" s="25"/>
-      <c r="B18" s="33"/>
-      <c r="C18" s="27"/>
-      <c r="D18" s="30"/>
-      <c r="E18" s="30"/>
+      <c r="A18" s="24"/>
+      <c r="B18" s="32"/>
+      <c r="C18" s="26"/>
+      <c r="D18" s="29"/>
+      <c r="E18" s="29"/>
       <c r="F18" s="10">
         <v>3</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I18" s="3" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>216</v>
-      </c>
-      <c r="M18" s="24"/>
+        <v>212</v>
+      </c>
+      <c r="K18" s="43"/>
+      <c r="L18" s="29"/>
+      <c r="M18" s="23"/>
       <c r="N18" s="9"/>
-      <c r="O18" s="34"/>
+      <c r="O18" s="35"/>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A19" s="25"/>
-      <c r="B19" s="18"/>
-      <c r="C19" s="19"/>
-      <c r="D19" s="19"/>
-      <c r="E19" s="19"/>
-      <c r="F19" s="19"/>
-      <c r="G19" s="19"/>
-      <c r="H19" s="19"/>
-      <c r="I19" s="19"/>
-      <c r="J19" s="20"/>
-      <c r="M19" s="24"/>
+      <c r="A19" s="24"/>
+      <c r="B19" s="21"/>
+      <c r="C19" s="22"/>
+      <c r="D19" s="22"/>
+      <c r="E19" s="22"/>
+      <c r="F19" s="22"/>
+      <c r="G19" s="22"/>
+      <c r="H19" s="22"/>
+      <c r="I19" s="22"/>
+      <c r="J19" s="22"/>
+      <c r="K19" s="22"/>
+      <c r="L19" s="46"/>
+      <c r="M19" s="23"/>
       <c r="N19" s="4"/>
-      <c r="O19" s="34"/>
+      <c r="O19" s="35"/>
     </row>
     <row r="20" spans="1:15" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A20" s="25" t="s">
+      <c r="A20" s="24" t="s">
         <v>31</v>
       </c>
-      <c r="B20" s="36" t="s">
+      <c r="B20" s="34" t="s">
         <v>14</v>
       </c>
-      <c r="C20" s="27" t="s">
+      <c r="C20" s="26" t="s">
         <v>26</v>
       </c>
-      <c r="D20" s="26" t="s">
+      <c r="D20" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="E20" s="26" t="s">
+      <c r="E20" s="25" t="s">
         <v>34</v>
       </c>
       <c r="F20" s="10">
         <v>1</v>
       </c>
       <c r="G20" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="H20" s="19" t="s">
+        <v>166</v>
+      </c>
+      <c r="I20" s="19" t="s">
         <v>167</v>
       </c>
-      <c r="H20" s="3" t="s">
+      <c r="J20" s="19" t="s">
         <v>168</v>
       </c>
-      <c r="I20" s="3" t="s">
-        <v>169</v>
-      </c>
-      <c r="J20" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="N20" s="34"/>
+      <c r="K20" s="41">
+        <v>8</v>
+      </c>
+      <c r="L20" s="27" t="s">
+        <v>244</v>
+      </c>
+      <c r="N20" s="35"/>
     </row>
     <row r="21" spans="1:15" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A21" s="25"/>
-      <c r="B21" s="36"/>
-      <c r="C21" s="27"/>
-      <c r="D21" s="26"/>
-      <c r="E21" s="26"/>
+      <c r="A21" s="24"/>
+      <c r="B21" s="34"/>
+      <c r="C21" s="26"/>
+      <c r="D21" s="25"/>
+      <c r="E21" s="25"/>
       <c r="F21" s="10">
         <v>2</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="H21" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="H21" s="19" t="s">
+        <v>169</v>
+      </c>
+      <c r="I21" s="19" t="s">
+        <v>170</v>
+      </c>
+      <c r="J21" s="19" t="s">
         <v>171</v>
       </c>
-      <c r="I21" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="J21" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="N21" s="34"/>
+      <c r="K21" s="42"/>
+      <c r="L21" s="28"/>
+      <c r="N21" s="35"/>
     </row>
     <row r="22" spans="1:15" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A22" s="25"/>
-      <c r="B22" s="36"/>
-      <c r="C22" s="27"/>
-      <c r="D22" s="26"/>
-      <c r="E22" s="26"/>
+      <c r="A22" s="24"/>
+      <c r="B22" s="34"/>
+      <c r="C22" s="26"/>
+      <c r="D22" s="25"/>
+      <c r="E22" s="25"/>
       <c r="F22" s="10">
         <v>3</v>
       </c>
       <c r="G22" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="H22" s="19" t="s">
+        <v>174</v>
+      </c>
+      <c r="I22" s="19" t="s">
         <v>175</v>
       </c>
-      <c r="H22" s="3" t="s">
+      <c r="J22" s="20" t="s">
         <v>176</v>
       </c>
-      <c r="I22" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="J22" s="11" t="s">
-        <v>178</v>
-      </c>
-      <c r="M22" s="24"/>
-      <c r="N22" s="34"/>
-      <c r="O22" s="34"/>
+      <c r="K22" s="43"/>
+      <c r="L22" s="29"/>
+      <c r="M22" s="23"/>
+      <c r="N22" s="35"/>
+      <c r="O22" s="35"/>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A23" s="25"/>
-      <c r="B23" s="18"/>
-      <c r="C23" s="19"/>
-      <c r="D23" s="19"/>
-      <c r="E23" s="19"/>
-      <c r="F23" s="19"/>
-      <c r="G23" s="19"/>
-      <c r="H23" s="19"/>
-      <c r="I23" s="19"/>
-      <c r="J23" s="20"/>
-      <c r="M23" s="24"/>
+      <c r="A23" s="24"/>
+      <c r="B23" s="21"/>
+      <c r="C23" s="22"/>
+      <c r="D23" s="22"/>
+      <c r="E23" s="22"/>
+      <c r="F23" s="22"/>
+      <c r="G23" s="22"/>
+      <c r="H23" s="22"/>
+      <c r="I23" s="22"/>
+      <c r="J23" s="22"/>
+      <c r="K23" s="22"/>
+      <c r="L23" s="46"/>
+      <c r="M23" s="23"/>
       <c r="N23" s="4"/>
-      <c r="O23" s="34"/>
+      <c r="O23" s="35"/>
     </row>
     <row r="24" spans="1:15" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A24" s="25"/>
-      <c r="B24" s="36" t="s">
+      <c r="A24" s="24"/>
+      <c r="B24" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="C24" s="27" t="s">
+      <c r="C24" s="26" t="s">
         <v>26</v>
       </c>
-      <c r="D24" s="26" t="s">
+      <c r="D24" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="E24" s="26" t="s">
+      <c r="E24" s="25" t="s">
         <v>38</v>
       </c>
       <c r="F24" s="10">
         <v>1</v>
       </c>
       <c r="G24" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="H24" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="H24" s="3" t="s">
+      <c r="I24" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="I24" s="3" t="s">
+      <c r="J24" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="J24" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="M24" s="24"/>
-      <c r="N24" s="34"/>
-      <c r="O24" s="34"/>
+      <c r="K24" s="41">
+        <v>3</v>
+      </c>
+      <c r="L24" s="27" t="s">
+        <v>245</v>
+      </c>
+      <c r="M24" s="23"/>
+      <c r="N24" s="35"/>
+      <c r="O24" s="35"/>
     </row>
     <row r="25" spans="1:15" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A25" s="25"/>
-      <c r="B25" s="36"/>
-      <c r="C25" s="27"/>
-      <c r="D25" s="26"/>
-      <c r="E25" s="26"/>
+      <c r="A25" s="24"/>
+      <c r="B25" s="34"/>
+      <c r="C25" s="26"/>
+      <c r="D25" s="25"/>
+      <c r="E25" s="25"/>
       <c r="F25" s="10">
         <v>2</v>
       </c>
       <c r="G25" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="H25" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="H25" s="3" t="s">
+      <c r="I25" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="J25" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="I25" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="J25" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="N25" s="34"/>
+      <c r="K25" s="42"/>
+      <c r="L25" s="28"/>
+      <c r="N25" s="35"/>
     </row>
     <row r="26" spans="1:15" ht="62.4" x14ac:dyDescent="0.3">
-      <c r="A26" s="25"/>
-      <c r="B26" s="36"/>
-      <c r="C26" s="27"/>
-      <c r="D26" s="26"/>
-      <c r="E26" s="26"/>
+      <c r="A26" s="24"/>
+      <c r="B26" s="34"/>
+      <c r="C26" s="26"/>
+      <c r="D26" s="25"/>
+      <c r="E26" s="25"/>
       <c r="F26" s="10">
         <v>3</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>218</v>
-      </c>
-      <c r="H26" s="16" t="s">
-        <v>219</v>
+        <v>214</v>
+      </c>
+      <c r="H26" s="3" t="s">
+        <v>215</v>
       </c>
       <c r="I26" s="3" t="s">
-        <v>221</v>
-      </c>
-      <c r="J26" s="17" t="s">
-        <v>220</v>
-      </c>
-      <c r="M26" s="24"/>
-      <c r="N26" s="34"/>
-      <c r="O26" s="34"/>
+        <v>217</v>
+      </c>
+      <c r="J26" s="15" t="s">
+        <v>216</v>
+      </c>
+      <c r="K26" s="43"/>
+      <c r="L26" s="29"/>
+      <c r="M26" s="23"/>
+      <c r="N26" s="35"/>
+      <c r="O26" s="35"/>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A27" s="25"/>
-      <c r="B27" s="18"/>
-      <c r="C27" s="19"/>
-      <c r="D27" s="19"/>
-      <c r="E27" s="19"/>
-      <c r="F27" s="19"/>
-      <c r="G27" s="19"/>
-      <c r="H27" s="19"/>
-      <c r="I27" s="19"/>
-      <c r="J27" s="20"/>
-      <c r="M27" s="24"/>
+      <c r="A27" s="24"/>
+      <c r="B27" s="21"/>
+      <c r="C27" s="22"/>
+      <c r="D27" s="22"/>
+      <c r="E27" s="22"/>
+      <c r="F27" s="22"/>
+      <c r="G27" s="22"/>
+      <c r="H27" s="22"/>
+      <c r="I27" s="22"/>
+      <c r="J27" s="22"/>
+      <c r="K27" s="22"/>
+      <c r="L27" s="46"/>
+      <c r="M27" s="23"/>
       <c r="N27" s="4"/>
-      <c r="O27" s="34"/>
+      <c r="O27" s="35"/>
     </row>
     <row r="28" spans="1:15" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A28" s="25" t="s">
+      <c r="A28" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="B28" s="36" t="s">
+      <c r="B28" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="C28" s="27" t="s">
+      <c r="C28" s="26" t="s">
         <v>40</v>
       </c>
-      <c r="D28" s="26" t="s">
+      <c r="D28" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="E28" s="26" t="s">
+      <c r="E28" s="25" t="s">
         <v>42</v>
       </c>
       <c r="F28" s="10">
         <v>1</v>
       </c>
       <c r="G28" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="H28" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="H28" s="3" t="s">
+      <c r="I28" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="J28" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="I28" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="J28" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="M28" s="24"/>
-      <c r="N28" s="34"/>
-      <c r="O28" s="34"/>
+      <c r="K28" s="41">
+        <v>3</v>
+      </c>
+      <c r="L28" s="27" t="s">
+        <v>246</v>
+      </c>
+      <c r="M28" s="23"/>
+      <c r="N28" s="35"/>
+      <c r="O28" s="35"/>
     </row>
     <row r="29" spans="1:15" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A29" s="25"/>
-      <c r="B29" s="36"/>
-      <c r="C29" s="27"/>
-      <c r="D29" s="26"/>
-      <c r="E29" s="26"/>
+      <c r="A29" s="24"/>
+      <c r="B29" s="34"/>
+      <c r="C29" s="26"/>
+      <c r="D29" s="25"/>
+      <c r="E29" s="25"/>
       <c r="F29" s="10">
         <v>2</v>
       </c>
       <c r="G29" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="H29" s="19" t="s">
+        <v>93</v>
+      </c>
+      <c r="I29" s="19" t="s">
         <v>179</v>
       </c>
-      <c r="H29" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="I29" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="J29" s="3" t="s">
-        <v>182</v>
-      </c>
-      <c r="N29" s="34"/>
+      <c r="J29" s="19" t="s">
+        <v>180</v>
+      </c>
+      <c r="K29" s="42"/>
+      <c r="L29" s="28"/>
+      <c r="N29" s="35"/>
     </row>
     <row r="30" spans="1:15" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A30" s="25"/>
-      <c r="B30" s="36"/>
-      <c r="C30" s="27"/>
-      <c r="D30" s="26"/>
-      <c r="E30" s="26"/>
+      <c r="A30" s="24"/>
+      <c r="B30" s="34"/>
+      <c r="C30" s="26"/>
+      <c r="D30" s="25"/>
+      <c r="E30" s="25"/>
       <c r="F30" s="10">
         <v>3</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>180</v>
-      </c>
-      <c r="H30" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="H30" s="19" t="s">
+        <v>181</v>
+      </c>
+      <c r="I30" s="19" t="s">
+        <v>182</v>
+      </c>
+      <c r="J30" s="19" t="s">
         <v>183</v>
       </c>
-      <c r="I30" s="3" t="s">
-        <v>184</v>
-      </c>
-      <c r="J30" s="3" t="s">
-        <v>185</v>
-      </c>
-      <c r="N30" s="34"/>
+      <c r="K30" s="43"/>
+      <c r="L30" s="29"/>
+      <c r="N30" s="35"/>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A31" s="25"/>
-      <c r="B31" s="18"/>
-      <c r="C31" s="19"/>
-      <c r="D31" s="19"/>
-      <c r="E31" s="19"/>
-      <c r="F31" s="19"/>
-      <c r="G31" s="19"/>
-      <c r="H31" s="19"/>
-      <c r="I31" s="19"/>
-      <c r="J31" s="20"/>
+      <c r="A31" s="24"/>
+      <c r="B31" s="21"/>
+      <c r="C31" s="22"/>
+      <c r="D31" s="22"/>
+      <c r="E31" s="22"/>
+      <c r="F31" s="22"/>
+      <c r="G31" s="22"/>
+      <c r="H31" s="22"/>
+      <c r="I31" s="22"/>
+      <c r="J31" s="22"/>
+      <c r="K31" s="22"/>
+      <c r="L31" s="46"/>
       <c r="N31" s="4"/>
     </row>
     <row r="32" spans="1:15" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A32" s="25"/>
-      <c r="B32" s="36" t="s">
+      <c r="A32" s="24"/>
+      <c r="B32" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="C32" s="27" t="s">
+      <c r="C32" s="26" t="s">
         <v>40</v>
       </c>
-      <c r="D32" s="26" t="s">
-        <v>111</v>
-      </c>
-      <c r="E32" s="26" t="s">
+      <c r="D32" s="25" t="s">
+        <v>110</v>
+      </c>
+      <c r="E32" s="25" t="s">
         <v>43</v>
       </c>
       <c r="F32" s="10">
         <v>1</v>
       </c>
       <c r="G32" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="H32" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="H32" s="3" t="s">
+      <c r="I32" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="I32" s="3" t="s">
+      <c r="J32" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="J32" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="M32" s="37"/>
-      <c r="N32" s="37"/>
-      <c r="O32" s="37"/>
+      <c r="K32" s="41">
+        <v>3</v>
+      </c>
+      <c r="L32" s="27" t="s">
+        <v>247</v>
+      </c>
+      <c r="M32" s="36"/>
+      <c r="N32" s="36"/>
+      <c r="O32" s="36"/>
     </row>
     <row r="33" spans="1:14" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A33" s="25"/>
-      <c r="B33" s="36"/>
-      <c r="C33" s="27"/>
-      <c r="D33" s="26"/>
-      <c r="E33" s="26"/>
+      <c r="A33" s="24"/>
+      <c r="B33" s="34"/>
+      <c r="C33" s="26"/>
+      <c r="D33" s="25"/>
+      <c r="E33" s="25"/>
       <c r="F33" s="10">
         <v>2</v>
       </c>
       <c r="G33" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="H33" s="19" t="s">
+        <v>185</v>
+      </c>
+      <c r="I33" s="19" t="s">
         <v>186</v>
       </c>
-      <c r="H33" s="3" t="s">
+      <c r="J33" s="19" t="s">
         <v>187</v>
       </c>
-      <c r="I33" s="3" t="s">
-        <v>188</v>
-      </c>
-      <c r="J33" s="3" t="s">
-        <v>189</v>
-      </c>
-      <c r="M33" s="15"/>
+      <c r="K33" s="42"/>
+      <c r="L33" s="28"/>
+      <c r="M33" s="14"/>
     </row>
     <row r="34" spans="1:14" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A34" s="25"/>
-      <c r="B34" s="36"/>
-      <c r="C34" s="27"/>
-      <c r="D34" s="26"/>
-      <c r="E34" s="26"/>
+      <c r="A34" s="24"/>
+      <c r="B34" s="34"/>
+      <c r="C34" s="26"/>
+      <c r="D34" s="25"/>
+      <c r="E34" s="25"/>
       <c r="F34" s="10">
         <v>3</v>
       </c>
       <c r="G34" s="11" t="s">
-        <v>217</v>
-      </c>
-      <c r="H34" s="3" t="s">
-        <v>187</v>
-      </c>
-      <c r="I34" s="3" t="s">
-        <v>203</v>
-      </c>
-      <c r="J34" s="3" t="s">
-        <v>204</v>
-      </c>
-      <c r="M34" s="15"/>
+        <v>213</v>
+      </c>
+      <c r="H34" s="19" t="s">
+        <v>185</v>
+      </c>
+      <c r="I34" s="19" t="s">
+        <v>199</v>
+      </c>
+      <c r="J34" s="19" t="s">
+        <v>200</v>
+      </c>
+      <c r="K34" s="43"/>
+      <c r="L34" s="29"/>
+      <c r="M34" s="14"/>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A35" s="25"/>
-      <c r="B35" s="18"/>
-      <c r="C35" s="19"/>
-      <c r="D35" s="19"/>
-      <c r="E35" s="19"/>
-      <c r="F35" s="19"/>
-      <c r="G35" s="19"/>
-      <c r="H35" s="19"/>
-      <c r="I35" s="19"/>
-      <c r="J35" s="20"/>
-      <c r="M35" s="15"/>
+      <c r="A35" s="24"/>
+      <c r="B35" s="21"/>
+      <c r="C35" s="22"/>
+      <c r="D35" s="22"/>
+      <c r="E35" s="22"/>
+      <c r="F35" s="22"/>
+      <c r="G35" s="22"/>
+      <c r="H35" s="22"/>
+      <c r="I35" s="22"/>
+      <c r="J35" s="22"/>
+      <c r="K35" s="22"/>
+      <c r="L35" s="46"/>
+      <c r="M35" s="14"/>
       <c r="N35" s="4"/>
     </row>
     <row r="36" spans="1:14" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A36" s="25"/>
-      <c r="B36" s="36" t="s">
+      <c r="A36" s="24"/>
+      <c r="B36" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="C36" s="27" t="s">
+      <c r="C36" s="26" t="s">
         <v>40</v>
       </c>
-      <c r="D36" s="26" t="s">
-        <v>112</v>
-      </c>
-      <c r="E36" s="26" t="s">
+      <c r="D36" s="25" t="s">
+        <v>111</v>
+      </c>
+      <c r="E36" s="25" t="s">
         <v>44</v>
       </c>
       <c r="F36" s="10">
         <v>1</v>
       </c>
       <c r="G36" s="3" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="H36" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="I36" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="I36" s="3" t="s">
+      <c r="J36" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="J36" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="N36" s="34"/>
-    </row>
-    <row r="37" spans="1:14" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A37" s="25"/>
-      <c r="B37" s="36"/>
-      <c r="C37" s="27"/>
-      <c r="D37" s="26"/>
-      <c r="E37" s="26"/>
+      <c r="K36" s="41">
+        <v>5</v>
+      </c>
+      <c r="L36" s="27" t="s">
+        <v>248</v>
+      </c>
+      <c r="N36" s="35"/>
+    </row>
+    <row r="37" spans="1:14" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A37" s="24"/>
+      <c r="B37" s="34"/>
+      <c r="C37" s="26"/>
+      <c r="D37" s="25"/>
+      <c r="E37" s="25"/>
       <c r="F37" s="10">
         <v>2</v>
       </c>
       <c r="G37" s="3" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="H37" s="3" t="s">
-        <v>191</v>
+        <v>235</v>
       </c>
       <c r="I37" s="3" t="s">
-        <v>192</v>
+        <v>221</v>
       </c>
       <c r="J37" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="N37" s="34"/>
-    </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A38" s="25"/>
-      <c r="B38" s="36"/>
-      <c r="C38" s="27"/>
-      <c r="D38" s="26"/>
-      <c r="E38" s="26"/>
+        <v>189</v>
+      </c>
+      <c r="K37" s="42"/>
+      <c r="L37" s="28"/>
+      <c r="N37" s="35"/>
+    </row>
+    <row r="38" spans="1:14" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A38" s="24"/>
+      <c r="B38" s="34"/>
+      <c r="C38" s="26"/>
+      <c r="D38" s="25"/>
+      <c r="E38" s="25"/>
       <c r="F38" s="10">
         <v>3</v>
       </c>
-      <c r="G38" s="14"/>
-      <c r="H38" s="3"/>
-      <c r="I38" s="3"/>
-      <c r="J38" s="3"/>
-      <c r="N38" s="34"/>
+      <c r="G38" s="18" t="s">
+        <v>223</v>
+      </c>
+      <c r="H38" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="I38" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="J38" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="K38" s="43"/>
+      <c r="L38" s="29"/>
+      <c r="N38" s="35"/>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A39" s="25"/>
-      <c r="B39" s="18"/>
-      <c r="C39" s="19"/>
-      <c r="D39" s="19"/>
-      <c r="E39" s="19"/>
-      <c r="F39" s="19"/>
-      <c r="G39" s="19"/>
-      <c r="H39" s="19"/>
-      <c r="I39" s="19"/>
-      <c r="J39" s="20"/>
+      <c r="A39" s="24"/>
+      <c r="B39" s="21"/>
+      <c r="C39" s="22"/>
+      <c r="D39" s="22"/>
+      <c r="E39" s="22"/>
+      <c r="F39" s="22"/>
+      <c r="G39" s="22"/>
+      <c r="H39" s="22"/>
+      <c r="I39" s="22"/>
+      <c r="J39" s="22"/>
+      <c r="K39" s="22"/>
+      <c r="L39" s="46"/>
       <c r="N39" s="4"/>
     </row>
     <row r="40" spans="1:14" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A40" s="25" t="s">
+      <c r="A40" s="24" t="s">
         <v>45</v>
       </c>
-      <c r="B40" s="36" t="s">
+      <c r="B40" s="34" t="s">
         <v>19</v>
       </c>
-      <c r="C40" s="27" t="s">
+      <c r="C40" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="D40" s="26" t="s">
+      <c r="D40" s="25" t="s">
         <v>47</v>
       </c>
-      <c r="E40" s="26" t="s">
+      <c r="E40" s="25" t="s">
         <v>48</v>
       </c>
       <c r="F40" s="10">
         <v>1</v>
       </c>
       <c r="G40" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="H40" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="H40" s="3" t="s">
+      <c r="I40" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="I40" s="3" t="s">
+      <c r="J40" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="J40" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="N40" s="34"/>
+      <c r="K40" s="41">
+        <v>8</v>
+      </c>
+      <c r="L40" s="27" t="s">
+        <v>249</v>
+      </c>
+      <c r="N40" s="35"/>
     </row>
     <row r="41" spans="1:14" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A41" s="25"/>
-      <c r="B41" s="36"/>
-      <c r="C41" s="27"/>
-      <c r="D41" s="26"/>
-      <c r="E41" s="26"/>
+      <c r="A41" s="24"/>
+      <c r="B41" s="34"/>
+      <c r="C41" s="26"/>
+      <c r="D41" s="25"/>
+      <c r="E41" s="25"/>
       <c r="F41" s="10">
         <v>2</v>
       </c>
       <c r="G41" s="3" t="s">
-        <v>194</v>
-      </c>
-      <c r="H41" s="3" t="s">
-        <v>195</v>
-      </c>
-      <c r="I41" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="J41" s="3" t="s">
-        <v>182</v>
-      </c>
-      <c r="N41" s="34"/>
-    </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A42" s="25"/>
-      <c r="B42" s="36"/>
-      <c r="C42" s="27"/>
-      <c r="D42" s="26"/>
-      <c r="E42" s="26"/>
+        <v>190</v>
+      </c>
+      <c r="H41" s="19" t="s">
+        <v>191</v>
+      </c>
+      <c r="I41" s="19" t="s">
+        <v>179</v>
+      </c>
+      <c r="J41" s="19" t="s">
+        <v>180</v>
+      </c>
+      <c r="K41" s="42"/>
+      <c r="L41" s="28"/>
+      <c r="N41" s="35"/>
+    </row>
+    <row r="42" spans="1:14" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A42" s="24"/>
+      <c r="B42" s="34"/>
+      <c r="C42" s="26"/>
+      <c r="D42" s="25"/>
+      <c r="E42" s="25"/>
       <c r="F42" s="10">
         <v>3</v>
       </c>
-      <c r="G42" s="14"/>
-      <c r="H42" s="3"/>
-      <c r="I42" s="3"/>
-      <c r="J42" s="3"/>
-      <c r="N42" s="34"/>
+      <c r="G42" s="18" t="s">
+        <v>226</v>
+      </c>
+      <c r="H42" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="I42" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="J42" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="K42" s="43"/>
+      <c r="L42" s="29"/>
+      <c r="N42" s="35"/>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A43" s="25"/>
-      <c r="B43" s="18"/>
-      <c r="C43" s="19"/>
-      <c r="D43" s="19"/>
-      <c r="E43" s="19"/>
-      <c r="F43" s="19"/>
-      <c r="G43" s="19"/>
-      <c r="H43" s="19"/>
-      <c r="I43" s="19"/>
-      <c r="J43" s="20"/>
+      <c r="A43" s="24"/>
+      <c r="B43" s="21"/>
+      <c r="C43" s="22"/>
+      <c r="D43" s="22"/>
+      <c r="E43" s="22"/>
+      <c r="F43" s="22"/>
+      <c r="G43" s="22"/>
+      <c r="H43" s="22"/>
+      <c r="I43" s="22"/>
+      <c r="J43" s="22"/>
+      <c r="K43" s="22"/>
+      <c r="L43" s="46"/>
       <c r="N43" s="4"/>
     </row>
     <row r="44" spans="1:14" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A44" s="25"/>
-      <c r="B44" s="36" t="s">
+      <c r="A44" s="24"/>
+      <c r="B44" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="C44" s="27" t="s">
+      <c r="C44" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="D44" s="26" t="s">
+      <c r="D44" s="25" t="s">
         <v>49</v>
       </c>
-      <c r="E44" s="26" t="s">
+      <c r="E44" s="25" t="s">
         <v>50</v>
       </c>
       <c r="F44" s="10">
         <v>1</v>
       </c>
       <c r="G44" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="H44" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="H44" s="3" t="s">
+      <c r="I44" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="I44" s="3" t="s">
+      <c r="J44" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="J44" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="N44" s="34"/>
+      <c r="K44" s="41">
+        <v>8</v>
+      </c>
+      <c r="L44" s="27" t="s">
+        <v>250</v>
+      </c>
+      <c r="N44" s="35"/>
     </row>
     <row r="45" spans="1:14" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A45" s="25"/>
-      <c r="B45" s="36"/>
-      <c r="C45" s="27"/>
-      <c r="D45" s="26"/>
-      <c r="E45" s="26"/>
+      <c r="A45" s="24"/>
+      <c r="B45" s="34"/>
+      <c r="C45" s="26"/>
+      <c r="D45" s="25"/>
+      <c r="E45" s="25"/>
       <c r="F45" s="10">
         <v>2</v>
       </c>
       <c r="G45" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="H45" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="H45" s="3" t="s">
+      <c r="I45" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="I45" s="3" t="s">
+      <c r="J45" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="J45" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="N45" s="34"/>
+      <c r="K45" s="42"/>
+      <c r="L45" s="28"/>
+      <c r="N45" s="35"/>
     </row>
     <row r="46" spans="1:14" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A46" s="25"/>
-      <c r="B46" s="36"/>
-      <c r="C46" s="27"/>
-      <c r="D46" s="26"/>
-      <c r="E46" s="26"/>
+      <c r="A46" s="24"/>
+      <c r="B46" s="34"/>
+      <c r="C46" s="26"/>
+      <c r="D46" s="25"/>
+      <c r="E46" s="25"/>
       <c r="F46" s="10">
         <v>3</v>
       </c>
       <c r="G46" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="H46" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="H46" s="3" t="s">
+      <c r="I46" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="I46" s="3" t="s">
+      <c r="J46" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="J46" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="N46" s="34"/>
+      <c r="K46" s="43"/>
+      <c r="L46" s="29"/>
+      <c r="N46" s="35"/>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A47" s="25"/>
-      <c r="B47" s="18"/>
-      <c r="C47" s="19"/>
-      <c r="D47" s="19"/>
-      <c r="E47" s="19"/>
-      <c r="F47" s="19"/>
-      <c r="G47" s="19"/>
-      <c r="H47" s="19"/>
-      <c r="I47" s="19"/>
-      <c r="J47" s="20"/>
+      <c r="A47" s="24"/>
+      <c r="B47" s="21"/>
+      <c r="C47" s="22"/>
+      <c r="D47" s="22"/>
+      <c r="E47" s="22"/>
+      <c r="F47" s="22"/>
+      <c r="G47" s="22"/>
+      <c r="H47" s="22"/>
+      <c r="I47" s="22"/>
+      <c r="J47" s="22"/>
+      <c r="K47" s="22"/>
+      <c r="L47" s="46"/>
       <c r="N47" s="4"/>
     </row>
     <row r="48" spans="1:14" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A48" s="25" t="s">
+      <c r="A48" s="24" t="s">
         <v>51</v>
       </c>
-      <c r="B48" s="36" t="s">
+      <c r="B48" s="34" t="s">
         <v>21</v>
       </c>
-      <c r="C48" s="27" t="s">
+      <c r="C48" s="26" t="s">
         <v>54</v>
       </c>
-      <c r="D48" s="26" t="s">
+      <c r="D48" s="25" t="s">
         <v>52</v>
       </c>
-      <c r="E48" s="26" t="s">
+      <c r="E48" s="25" t="s">
         <v>53</v>
       </c>
       <c r="F48" s="10">
         <v>1</v>
       </c>
       <c r="G48" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="H48" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="H48" s="3" t="s">
+      <c r="I48" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="I48" s="3" t="s">
+      <c r="J48" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="J48" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="N48" s="34"/>
+      <c r="K48" s="41">
+        <v>5</v>
+      </c>
+      <c r="L48" s="27" t="s">
+        <v>251</v>
+      </c>
+      <c r="N48" s="35"/>
     </row>
     <row r="49" spans="1:14" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A49" s="25"/>
-      <c r="B49" s="36"/>
-      <c r="C49" s="27"/>
-      <c r="D49" s="26"/>
-      <c r="E49" s="26"/>
+      <c r="A49" s="24"/>
+      <c r="B49" s="34"/>
+      <c r="C49" s="26"/>
+      <c r="D49" s="25"/>
+      <c r="E49" s="25"/>
       <c r="F49" s="10">
         <v>2</v>
       </c>
       <c r="G49" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="H49" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="H49" s="3" t="s">
+      <c r="I49" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="J49" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="I49" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="J49" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="N49" s="34"/>
+      <c r="K49" s="42"/>
+      <c r="L49" s="28"/>
+      <c r="N49" s="35"/>
     </row>
     <row r="50" spans="1:14" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A50" s="25"/>
-      <c r="B50" s="36"/>
-      <c r="C50" s="27"/>
-      <c r="D50" s="26"/>
-      <c r="E50" s="26"/>
+      <c r="A50" s="24"/>
+      <c r="B50" s="34"/>
+      <c r="C50" s="26"/>
+      <c r="D50" s="25"/>
+      <c r="E50" s="25"/>
       <c r="F50" s="10">
         <v>3</v>
       </c>
       <c r="G50" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="H50" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="H50" s="3" t="s">
+      <c r="I50" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="J50" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="I50" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="J50" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="N50" s="34"/>
+      <c r="K50" s="43"/>
+      <c r="L50" s="29"/>
+      <c r="N50" s="35"/>
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A51" s="25"/>
-      <c r="B51" s="18"/>
-      <c r="C51" s="19"/>
-      <c r="D51" s="19"/>
-      <c r="E51" s="19"/>
-      <c r="F51" s="19"/>
-      <c r="G51" s="19"/>
-      <c r="H51" s="19"/>
-      <c r="I51" s="19"/>
-      <c r="J51" s="20"/>
+      <c r="A51" s="24"/>
+      <c r="B51" s="21"/>
+      <c r="C51" s="22"/>
+      <c r="D51" s="22"/>
+      <c r="E51" s="22"/>
+      <c r="F51" s="22"/>
+      <c r="G51" s="22"/>
+      <c r="H51" s="22"/>
+      <c r="I51" s="22"/>
+      <c r="J51" s="22"/>
+      <c r="K51" s="22"/>
+      <c r="L51" s="46"/>
       <c r="N51" s="4"/>
     </row>
     <row r="52" spans="1:14" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A52" s="25"/>
-      <c r="B52" s="36" t="s">
+      <c r="A52" s="24"/>
+      <c r="B52" s="34" t="s">
         <v>22</v>
       </c>
-      <c r="C52" s="27" t="s">
+      <c r="C52" s="26" t="s">
         <v>54</v>
       </c>
-      <c r="D52" s="26" t="s">
+      <c r="D52" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="E52" s="26" t="s">
-        <v>196</v>
+      <c r="E52" s="25" t="s">
+        <v>192</v>
       </c>
       <c r="F52" s="10">
         <v>1</v>
       </c>
       <c r="G52" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="H52" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="I52" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="H52" s="3" t="s">
+      <c r="J52" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="I52" s="3" t="s">
-        <v>144</v>
-      </c>
-      <c r="J52" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="N52" s="34"/>
+      <c r="K52" s="41">
+        <v>8</v>
+      </c>
+      <c r="L52" s="27" t="s">
+        <v>252</v>
+      </c>
+      <c r="N52" s="35"/>
     </row>
     <row r="53" spans="1:14" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A53" s="25"/>
-      <c r="B53" s="36"/>
-      <c r="C53" s="27"/>
-      <c r="D53" s="26"/>
-      <c r="E53" s="26"/>
+      <c r="A53" s="24"/>
+      <c r="B53" s="34"/>
+      <c r="C53" s="26"/>
+      <c r="D53" s="25"/>
+      <c r="E53" s="25"/>
       <c r="F53" s="10">
         <v>2</v>
       </c>
       <c r="G53" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="H53" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="I53" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="H53" s="3" t="s">
+      <c r="J53" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="I53" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="J53" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="N53" s="34"/>
+      <c r="K53" s="42"/>
+      <c r="L53" s="28"/>
+      <c r="N53" s="35"/>
     </row>
     <row r="54" spans="1:14" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A54" s="25"/>
-      <c r="B54" s="36"/>
-      <c r="C54" s="27"/>
-      <c r="D54" s="26"/>
-      <c r="E54" s="26"/>
+      <c r="A54" s="24"/>
+      <c r="B54" s="34"/>
+      <c r="C54" s="26"/>
+      <c r="D54" s="25"/>
+      <c r="E54" s="25"/>
       <c r="F54" s="10">
         <v>3</v>
       </c>
       <c r="G54" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="H54" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="I54" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="J54" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="H54" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="I54" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="J54" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="N54" s="34"/>
+      <c r="K54" s="43"/>
+      <c r="L54" s="29"/>
+      <c r="N54" s="35"/>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A55" s="25"/>
-      <c r="B55" s="18"/>
-      <c r="C55" s="19"/>
-      <c r="D55" s="19"/>
-      <c r="E55" s="19"/>
-      <c r="F55" s="19"/>
-      <c r="G55" s="19"/>
-      <c r="H55" s="19"/>
-      <c r="I55" s="19"/>
-      <c r="J55" s="20"/>
+      <c r="A55" s="24"/>
+      <c r="B55" s="21"/>
+      <c r="C55" s="22"/>
+      <c r="D55" s="22"/>
+      <c r="E55" s="22"/>
+      <c r="F55" s="22"/>
+      <c r="G55" s="22"/>
+      <c r="H55" s="22"/>
+      <c r="I55" s="22"/>
+      <c r="J55" s="22"/>
+      <c r="K55" s="22"/>
+      <c r="L55" s="46"/>
       <c r="N55" s="4"/>
     </row>
     <row r="56" spans="1:14" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A56" s="25"/>
-      <c r="B56" s="31" t="s">
+      <c r="A56" s="24"/>
+      <c r="B56" s="30" t="s">
         <v>23</v>
       </c>
-      <c r="C56" s="27" t="s">
+      <c r="C56" s="26" t="s">
         <v>54</v>
       </c>
-      <c r="D56" s="26" t="s">
+      <c r="D56" s="25" t="s">
         <v>57</v>
       </c>
-      <c r="E56" s="26" t="s">
+      <c r="E56" s="25" t="s">
         <v>56</v>
       </c>
       <c r="F56" s="10">
         <v>1</v>
       </c>
       <c r="G56" s="3" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="H56" s="3" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="I56" s="3" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="J56" s="3" t="s">
-        <v>163</v>
-      </c>
-      <c r="N56" s="34"/>
+        <v>161</v>
+      </c>
+      <c r="K56" s="41">
+        <v>8</v>
+      </c>
+      <c r="L56" s="27" t="s">
+        <v>253</v>
+      </c>
+      <c r="N56" s="35"/>
     </row>
     <row r="57" spans="1:14" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A57" s="25"/>
-      <c r="B57" s="32"/>
-      <c r="C57" s="27"/>
-      <c r="D57" s="26"/>
-      <c r="E57" s="26"/>
+      <c r="A57" s="24"/>
+      <c r="B57" s="31"/>
+      <c r="C57" s="26"/>
+      <c r="D57" s="25"/>
+      <c r="E57" s="25"/>
       <c r="F57" s="10">
         <v>2</v>
       </c>
       <c r="G57" s="13" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="H57" s="3" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="I57" s="3" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="J57" s="3" t="s">
-        <v>199</v>
-      </c>
-      <c r="N57" s="34"/>
+        <v>195</v>
+      </c>
+      <c r="K57" s="42"/>
+      <c r="L57" s="28"/>
+      <c r="N57" s="35"/>
     </row>
     <row r="58" spans="1:14" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A58" s="25"/>
-      <c r="B58" s="33"/>
-      <c r="C58" s="27"/>
-      <c r="D58" s="26"/>
-      <c r="E58" s="26"/>
+      <c r="A58" s="24"/>
+      <c r="B58" s="32"/>
+      <c r="C58" s="26"/>
+      <c r="D58" s="25"/>
+      <c r="E58" s="25"/>
       <c r="F58" s="10">
         <v>3</v>
       </c>
       <c r="G58" s="8" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="H58" s="3" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="I58" s="3" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="J58" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="N58" s="34"/>
+        <v>198</v>
+      </c>
+      <c r="K58" s="43"/>
+      <c r="L58" s="29"/>
+      <c r="N58" s="35"/>
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A59" s="25"/>
-      <c r="B59" s="18"/>
-      <c r="C59" s="19"/>
-      <c r="D59" s="19"/>
-      <c r="E59" s="19"/>
-      <c r="F59" s="19"/>
-      <c r="G59" s="19"/>
-      <c r="H59" s="19"/>
-      <c r="I59" s="19"/>
-      <c r="J59" s="20"/>
+      <c r="A59" s="24"/>
+      <c r="B59" s="21"/>
+      <c r="C59" s="22"/>
+      <c r="D59" s="22"/>
+      <c r="E59" s="22"/>
+      <c r="F59" s="22"/>
+      <c r="G59" s="22"/>
+      <c r="H59" s="22"/>
+      <c r="I59" s="22"/>
+      <c r="J59" s="22"/>
+      <c r="K59" s="22"/>
+      <c r="L59" s="46"/>
       <c r="N59" s="4"/>
     </row>
     <row r="60" spans="1:14" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A60" s="25" t="s">
-        <v>141</v>
-      </c>
-      <c r="B60" s="31" t="s">
+      <c r="A60" s="24" t="s">
+        <v>139</v>
+      </c>
+      <c r="B60" s="30" t="s">
         <v>24</v>
       </c>
-      <c r="C60" s="27" t="s">
+      <c r="C60" s="26" t="s">
         <v>26</v>
       </c>
-      <c r="D60" s="26" t="s">
-        <v>158</v>
-      </c>
-      <c r="E60" s="28" t="s">
+      <c r="D60" s="25" t="s">
+        <v>156</v>
+      </c>
+      <c r="E60" s="27" t="s">
         <v>58</v>
       </c>
       <c r="F60" s="10">
         <v>1</v>
       </c>
       <c r="G60" s="3" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="H60" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="I60" s="3" t="s">
         <v>157</v>
       </c>
-      <c r="I60" s="3" t="s">
-        <v>159</v>
-      </c>
       <c r="J60" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="N60" s="34"/>
-    </row>
-    <row r="61" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A61" s="25"/>
-      <c r="B61" s="32"/>
-      <c r="C61" s="27"/>
-      <c r="D61" s="26"/>
-      <c r="E61" s="29"/>
+        <v>158</v>
+      </c>
+      <c r="K60" s="41">
+        <v>5</v>
+      </c>
+      <c r="L60" s="27" t="s">
+        <v>254</v>
+      </c>
+      <c r="N60" s="35"/>
+    </row>
+    <row r="61" spans="1:14" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A61" s="24"/>
+      <c r="B61" s="31"/>
+      <c r="C61" s="26"/>
+      <c r="D61" s="25"/>
+      <c r="E61" s="28"/>
       <c r="F61" s="10">
         <v>2</v>
       </c>
-      <c r="G61" s="14"/>
-      <c r="H61" s="3"/>
-      <c r="I61" s="3"/>
-      <c r="J61" s="3"/>
-      <c r="N61" s="34"/>
-    </row>
-    <row r="62" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A62" s="25"/>
-      <c r="B62" s="33"/>
-      <c r="C62" s="27"/>
-      <c r="D62" s="26"/>
-      <c r="E62" s="30"/>
+      <c r="G61" s="18" t="s">
+        <v>218</v>
+      </c>
+      <c r="H61" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="I61" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="J61" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="K61" s="42"/>
+      <c r="L61" s="28"/>
+      <c r="N61" s="35"/>
+    </row>
+    <row r="62" spans="1:14" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A62" s="24"/>
+      <c r="B62" s="32"/>
+      <c r="C62" s="26"/>
+      <c r="D62" s="25"/>
+      <c r="E62" s="29"/>
       <c r="F62" s="10">
         <v>3</v>
       </c>
-      <c r="G62" s="14"/>
-      <c r="H62" s="3"/>
-      <c r="I62" s="3"/>
-      <c r="J62" s="3"/>
-      <c r="N62" s="34"/>
+      <c r="G62" s="18" t="s">
+        <v>230</v>
+      </c>
+      <c r="H62" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="I62" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="J62" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="K62" s="43"/>
+      <c r="L62" s="29"/>
+      <c r="N62" s="35"/>
     </row>
     <row r="63" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A63" s="25"/>
-      <c r="B63" s="18"/>
-      <c r="C63" s="19"/>
-      <c r="D63" s="19"/>
-      <c r="E63" s="19"/>
-      <c r="F63" s="19"/>
-      <c r="G63" s="19"/>
-      <c r="H63" s="19"/>
-      <c r="I63" s="19"/>
-      <c r="J63" s="20"/>
+      <c r="A63" s="24"/>
+      <c r="B63" s="21"/>
+      <c r="C63" s="22"/>
+      <c r="D63" s="22"/>
+      <c r="E63" s="22"/>
+      <c r="F63" s="22"/>
+      <c r="G63" s="22"/>
+      <c r="H63" s="22"/>
+      <c r="I63" s="22"/>
+      <c r="J63" s="22"/>
+      <c r="K63" s="22"/>
+      <c r="L63" s="46"/>
       <c r="N63" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="108">
-    <mergeCell ref="B31:J31"/>
+  <mergeCells count="139">
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="L40:L42"/>
+    <mergeCell ref="K40:K42"/>
+    <mergeCell ref="L36:L38"/>
+    <mergeCell ref="K36:K38"/>
+    <mergeCell ref="L32:L34"/>
+    <mergeCell ref="K32:K34"/>
+    <mergeCell ref="B7:L7"/>
+    <mergeCell ref="B11:L11"/>
+    <mergeCell ref="B15:L15"/>
+    <mergeCell ref="B19:L19"/>
+    <mergeCell ref="B23:L23"/>
+    <mergeCell ref="B27:L27"/>
+    <mergeCell ref="B31:L31"/>
+    <mergeCell ref="B35:L35"/>
+    <mergeCell ref="B39:L39"/>
+    <mergeCell ref="L60:L62"/>
+    <mergeCell ref="K60:K62"/>
+    <mergeCell ref="L56:L58"/>
+    <mergeCell ref="K56:K58"/>
+    <mergeCell ref="L52:L54"/>
+    <mergeCell ref="K52:K54"/>
+    <mergeCell ref="L48:L50"/>
+    <mergeCell ref="K48:K50"/>
+    <mergeCell ref="L44:L46"/>
+    <mergeCell ref="K44:K46"/>
+    <mergeCell ref="B47:L47"/>
+    <mergeCell ref="B51:L51"/>
+    <mergeCell ref="B55:L55"/>
+    <mergeCell ref="B59:L59"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="L28:L30"/>
+    <mergeCell ref="K28:K30"/>
+    <mergeCell ref="L24:L26"/>
+    <mergeCell ref="K24:K26"/>
+    <mergeCell ref="L20:L22"/>
+    <mergeCell ref="K20:K22"/>
+    <mergeCell ref="L16:L18"/>
+    <mergeCell ref="K16:K18"/>
+    <mergeCell ref="L12:L14"/>
+    <mergeCell ref="K12:K14"/>
+    <mergeCell ref="L8:L10"/>
+    <mergeCell ref="K8:K10"/>
+    <mergeCell ref="L4:L6"/>
+    <mergeCell ref="K4:K6"/>
     <mergeCell ref="N20:N22"/>
     <mergeCell ref="C24:C26"/>
     <mergeCell ref="D24:D26"/>
     <mergeCell ref="N24:N26"/>
     <mergeCell ref="E20:E22"/>
-    <mergeCell ref="E52:E54"/>
-    <mergeCell ref="E48:E50"/>
-    <mergeCell ref="E44:E46"/>
-    <mergeCell ref="B8:B10"/>
-    <mergeCell ref="B12:B14"/>
-    <mergeCell ref="B20:B22"/>
-    <mergeCell ref="B24:B26"/>
     <mergeCell ref="B28:B30"/>
     <mergeCell ref="B52:B54"/>
     <mergeCell ref="E24:E26"/>
@@ -2812,8 +3218,10 @@
     <mergeCell ref="B40:B42"/>
     <mergeCell ref="B44:B46"/>
     <mergeCell ref="B48:B50"/>
-    <mergeCell ref="B39:J39"/>
-    <mergeCell ref="B35:J35"/>
+    <mergeCell ref="E52:E54"/>
+    <mergeCell ref="E48:E50"/>
+    <mergeCell ref="E44:E46"/>
+    <mergeCell ref="B43:L43"/>
     <mergeCell ref="A28:A39"/>
     <mergeCell ref="A48:A59"/>
     <mergeCell ref="N56:N58"/>
@@ -2842,14 +3250,9 @@
     <mergeCell ref="D56:D58"/>
     <mergeCell ref="D60:D62"/>
     <mergeCell ref="A40:A47"/>
-    <mergeCell ref="B47:J47"/>
-    <mergeCell ref="B63:J63"/>
-    <mergeCell ref="B59:J59"/>
-    <mergeCell ref="B55:J55"/>
-    <mergeCell ref="B51:J51"/>
-    <mergeCell ref="B43:J43"/>
     <mergeCell ref="B60:B62"/>
     <mergeCell ref="E60:E62"/>
+    <mergeCell ref="B63:L63"/>
     <mergeCell ref="N60:N62"/>
     <mergeCell ref="E56:E58"/>
     <mergeCell ref="C32:C34"/>
@@ -2874,11 +3277,6 @@
     <mergeCell ref="D4:D6"/>
     <mergeCell ref="N4:N6"/>
     <mergeCell ref="E4:E6"/>
-    <mergeCell ref="B19:J19"/>
-    <mergeCell ref="B15:J15"/>
-    <mergeCell ref="B11:J11"/>
-    <mergeCell ref="B7:J7"/>
-    <mergeCell ref="A1:J1"/>
     <mergeCell ref="M9:M11"/>
     <mergeCell ref="M13:M19"/>
     <mergeCell ref="M22:M24"/>
@@ -2892,11 +3290,13 @@
     <mergeCell ref="D16:D18"/>
     <mergeCell ref="C16:C18"/>
     <mergeCell ref="B16:B18"/>
-    <mergeCell ref="B27:J27"/>
-    <mergeCell ref="B23:J23"/>
     <mergeCell ref="B2:E2"/>
     <mergeCell ref="F2:J2"/>
     <mergeCell ref="B4:B6"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="B12:B14"/>
+    <mergeCell ref="B20:B22"/>
+    <mergeCell ref="B24:B26"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>